<commit_message>
DSCW: propagate terminal growth revision (11.5% -> 5%) to the live site
- fair.full 1.29 -> 1.20 (bull-case DCF no longer clears the zero floor)
- CBE-rate lever recalibrated to the new sensitivity (impact 6.0 -> 4.2)
- study docx/xlsx/pdf refreshed with the full rebuild (all figures, §1.7
  disclosure of the anchor gap, Expert 3 branch convergence)
- noted, not fixed (pre-existing, unrelated): the CBE lever's min/max
  sign convention looks inverted vs the right=higher-value standard
</commit_message>
<xml_diff>
--- a/files/DSCW_Valuation_Study_19-07-2026_public.xlsx
+++ b/files/DSCW_Valuation_Study_19-07-2026_public.xlsx
@@ -758,7 +758,7 @@
     <t xml:space="preserve">vs spot</t>
   </si>
   <si>
-    <t xml:space="preserve">Scenario re-runs (compute.py): bear -1.02 · bull 0.33 · easing-path WACC 20.5% dual-frame -0.01 · market-implied WACC 16.07%</t>
+    <t xml:space="preserve">Scenario re-runs (compute.py): bear -0.94 · bull 0.06 · easing-path WACC 20.5% dual-frame -0.17 · market-implied WACC 13.05%</t>
   </si>
   <si>
     <t xml:space="preserve">Component</t>
@@ -896,7 +896,7 @@
     <t xml:space="preserve">FCFF DCF @ sourced WACC (floored at 0)</t>
   </si>
   <si>
-    <t xml:space="preserve">raw (unfloored): -1.02 / -0.50 / 0.33 — negative at today's rates, disclosed</t>
+    <t xml:space="preserve">raw (unfloored): -0.94 / -0.51 / 0.06 — negative at today's rates, disclosed</t>
   </si>
   <si>
     <t xml:space="preserve">Normalized earnings power</t>
@@ -917,7 +917,7 @@
     <t xml:space="preserve">weights must sum to 100%</t>
   </si>
   <si>
-    <t xml:space="preserve">Spot 1.94 sits above the bull central — at today's sourced cost of capital. The easing-path DCF (20.5% WACC: -0.01) and the market-implied WACC (16.1%) are the dual-framed reads of what the market is paying for; they are deliberately NOT blended into the central.</t>
+    <t xml:space="preserve">Spot 1.94 sits above the bull central — at today's sourced cost of capital. The easing-path DCF (20.5% WACC: -0.17) and the market-implied WACC (13.0%) are the dual-framed reads of what the market is paying for; they are deliberately NOT blended into the central.</t>
   </si>
   <si>
     <t xml:space="preserve">Item</t>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="B16" s="10" t="n">
         <f aca="false">F6*(1+Assumptions!$C$35)</f>
-        <v>1779.42789153843</v>
+        <v>1675.69442700928</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="B17" s="16" t="n">
         <f aca="false">Assumptions!$C$35/Assumptions!$C$36</f>
-        <v>0.522727272727273</v>
+        <v>0.227272727272727</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2302,7 +2302,7 @@
       </c>
       <c r="B18" s="14" t="n">
         <f aca="false">B16*(1-B17)/(B14-Assumptions!$C$35)</f>
-        <v>7061.82995095152</v>
+        <v>6989.30272849422</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="B19" s="22" t="n">
         <f aca="false">B18/(1+B14)^5</f>
-        <v>2455.39404516845</v>
+        <v>2430.17637335093</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="B20" s="22" t="n">
         <f aca="false">B15+B19</f>
-        <v>2623.05909304879</v>
+        <v>2597.84142123126</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="B21" s="16" t="n">
         <f aca="false">B19/B20</f>
-        <v>0.936080339049679</v>
+        <v>0.935459860440261</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="B24" s="22" t="n">
         <f aca="false">B20+B22+B23</f>
-        <v>-1345.14090695122</v>
+        <v>-1370.35857876874</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B25" s="24" t="n">
         <f aca="false">B24/Assumptions!$D$37</f>
-        <v>-0.501918248862394</v>
+        <v>-0.511327827898784</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="B26" s="16" t="n">
         <f aca="false">B25/Assumptions!$C$37-1</f>
-        <v>-1.25872074683629</v>
+        <v>-1.26357104530865</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2583,7 +2583,7 @@
         <v>0.224455466242559</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>-0.357784084027833</v>
+        <v>-0.403442993736621</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2599,7 +2599,7 @@
         <v>0.229858917862231</v>
       </c>
       <c r="D19" s="15" t="n">
-        <v>-0.433383166381358</v>
+        <v>-0.459212095708307</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2615,7 +2615,7 @@
         <v>0.235262369481904</v>
       </c>
       <c r="D20" s="15" t="n">
-        <v>-0.501918248862394</v>
+        <v>-0.511327827898784</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2631,7 +2631,7 @@
         <v>0.240665821101576</v>
       </c>
       <c r="D21" s="15" t="n">
-        <v>-0.564304894024218</v>
+        <v>-0.560110203111533</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2647,7 +2647,7 @@
         <v>0.246069272721248</v>
       </c>
       <c r="D22" s="15" t="n">
-        <v>-0.621307601859054</v>
+        <v>-0.605843684655369</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2663,7 +2663,7 @@
         <v>0.251472724340921</v>
       </c>
       <c r="D23" s="15" t="n">
-        <v>-0.673569717107819</v>
+        <v>-0.648781962754238</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2702,19 +2702,19 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="25" t="n">
-        <v>0.095</v>
+        <v>0.03</v>
       </c>
       <c r="C2" s="25" t="n">
-        <v>0.105</v>
+        <v>0.04</v>
       </c>
       <c r="D2" s="25" t="n">
-        <v>0.115</v>
+        <v>0.05</v>
       </c>
       <c r="E2" s="25" t="n">
-        <v>0.125</v>
+        <v>0.06</v>
       </c>
       <c r="F2" s="25" t="n">
-        <v>0.135</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2722,19 +2722,19 @@
         <v>0.205262369481904</v>
       </c>
       <c r="B3" s="15" t="n">
-        <v>-0.0723462295696986</v>
+        <v>-0.205105736952615</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>-0.0446042928383302</v>
+        <v>-0.187936729896757</v>
       </c>
       <c r="D3" s="15" t="n">
-        <v>-0.013073507021773</v>
+        <v>-0.169927004623318</v>
       </c>
       <c r="E3" s="15" t="n">
-        <v>0.0236623017767736</v>
+        <v>-0.150902933601524</v>
       </c>
       <c r="F3" s="15" t="n">
-        <v>0.0678255278575758</v>
+        <v>-0.130639543894947</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2742,19 +2742,19 @@
         <v>0.215262369481904</v>
       </c>
       <c r="B4" s="15" t="n">
-        <v>-0.239853340811866</v>
+        <v>-0.323381773877313</v>
       </c>
       <c r="C4" s="15" t="n">
-        <v>-0.22520788887397</v>
+        <v>-0.311359351993288</v>
       </c>
       <c r="D4" s="15" t="n">
-        <v>-0.209678005862878</v>
+        <v>-0.299117796412475</v>
       </c>
       <c r="E4" s="15" t="n">
-        <v>-0.192969738358711</v>
+        <v>-0.286614765832692</v>
       </c>
       <c r="F4" s="15" t="n">
-        <v>-0.174642636683486</v>
+        <v>-0.273796259689327</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2762,19 +2762,19 @@
         <v>0.225262369481904</v>
       </c>
       <c r="B5" s="15" t="n">
-        <v>-0.380366107130067</v>
+        <v>-0.427926721968106</v>
       </c>
       <c r="C5" s="15" t="n">
-        <v>-0.374598644423777</v>
+        <v>-0.419872053271118</v>
       </c>
       <c r="D5" s="15" t="n">
-        <v>-0.36956293882802</v>
+        <v>-0.412016749407447</v>
       </c>
       <c r="E5" s="15" t="n">
-        <v>-0.365477943010975</v>
+        <v>-0.404397000981273</v>
       </c>
       <c r="F5" s="15" t="n">
-        <v>-0.362659639075981</v>
+        <v>-0.397058322325194</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2782,19 +2782,19 @@
         <v>0.235262369481904</v>
       </c>
       <c r="B6" s="15" t="n">
-        <v>-0.499703543531874</v>
+        <v>-0.520818705342746</v>
       </c>
       <c r="C6" s="15" t="n">
-        <v>-0.500003394828182</v>
+        <v>-0.515834310553956</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>-0.501918248862394</v>
+        <v>-0.511327827898784</v>
       </c>
       <c r="E6" s="15" t="n">
-        <v>-0.505887512862604</v>
+        <v>-0.507381062524853</v>
       </c>
       <c r="F6" s="15" t="n">
-        <v>-0.512525897006701</v>
+        <v>-0.504095619646286</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2802,19 +2802,19 @@
         <v>0.245262369481904</v>
       </c>
       <c r="B7" s="15" t="n">
-        <v>-0.602133608442603</v>
+        <v>-0.60374586560344</v>
       </c>
       <c r="C7" s="15" t="n">
-        <v>-0.606586462456918</v>
+        <v>-0.601142160229424</v>
       </c>
       <c r="D7" s="15" t="n">
-        <v>-0.613110880181108</v>
+        <v>-0.599197647970579</v>
       </c>
       <c r="E7" s="15" t="n">
-        <v>-0.622223622689849</v>
+        <v>-0.598019073620844</v>
       </c>
       <c r="F7" s="15" t="n">
-        <v>-0.634628917036315</v>
+        <v>-0.597737544258947</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2822,19 +2822,19 @@
         <v>0.255262369481904</v>
       </c>
       <c r="B8" s="15" t="n">
-        <v>-0.690857223561919</v>
+        <v>-0.678093162085863</v>
       </c>
       <c r="C8" s="15" t="n">
-        <v>-0.698136036189027</v>
+        <v>-0.67733606854336</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>-0.707691143774233</v>
+        <v>-0.677351451716734</v>
       </c>
       <c r="E8" s="15" t="n">
-        <v>-0.720046787117198</v>
+        <v>-0.678257994491671</v>
       </c>
       <c r="F8" s="15" t="n">
-        <v>-0.735901572715487</v>
+        <v>-0.680200004576863</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2864,19 +2864,19 @@
         <v>266</v>
       </c>
       <c r="B12" s="15" t="n">
-        <v>-0.591486431073948</v>
+        <v>-0.668363365661827</v>
       </c>
       <c r="C12" s="15" t="n">
-        <v>-0.725451825413952</v>
+        <v>-0.761942505891463</v>
       </c>
       <c r="D12" s="15" t="n">
-        <v>-0.835862242322693</v>
+        <v>-0.843950136845197</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>-0.92818570865167</v>
+        <v>-0.91622675127954</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>-1.00632902832102</v>
+        <v>-0.980250897911853</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2884,19 +2884,19 @@
         <v>267</v>
       </c>
       <c r="B13" s="15" t="n">
-        <v>-0.400582218468414</v>
+        <v>-0.483740581037151</v>
       </c>
       <c r="C13" s="15" t="n">
-        <v>-0.547507382120987</v>
+        <v>-0.586979627649455</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>-0.668890245592544</v>
+        <v>-0.677638982371991</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>-0.770648294416389</v>
+        <v>-0.75771219962506</v>
       </c>
       <c r="F13" s="15" t="n">
-        <v>-0.857010086047625</v>
+        <v>-0.828801174814294</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2904,19 +2904,19 @@
         <v>268</v>
       </c>
       <c r="B14" s="15" t="n">
-        <v>-0.209678005862878</v>
+        <v>-0.299117796412475</v>
       </c>
       <c r="C14" s="15" t="n">
-        <v>-0.36956293882802</v>
+        <v>-0.412016749407447</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>-0.501918248862394</v>
+        <v>-0.511327827898784</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>-0.613110880181108</v>
+        <v>-0.599197647970579</v>
       </c>
       <c r="F14" s="15" t="n">
-        <v>-0.707691143774233</v>
+        <v>-0.677351451716734</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2924,19 +2924,19 @@
         <v>269</v>
       </c>
       <c r="B15" s="15" t="n">
-        <v>-0.0187737932573434</v>
+        <v>-0.114495011787798</v>
       </c>
       <c r="C15" s="15" t="n">
-        <v>-0.191618495535054</v>
+        <v>-0.237053871165439</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>-0.334946252132244</v>
+        <v>-0.345016673425577</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>-0.455573465945826</v>
+        <v>-0.440683096316097</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>-0.55837220150084</v>
+        <v>-0.525901728619174</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2944,19 +2944,19 @@
         <v>270</v>
       </c>
       <c r="B16" s="15" t="n">
-        <v>0.172130419348192</v>
+        <v>0.0701277728368787</v>
       </c>
       <c r="C16" s="15" t="n">
-        <v>-0.0136740522420876</v>
+        <v>-0.0620909929234304</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>-0.167974255402095</v>
+        <v>-0.17870551895237</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>-0.298036051710545</v>
+        <v>-0.282168544661616</v>
       </c>
       <c r="F16" s="15" t="n">
-        <v>-0.409053259227448</v>
+        <v>-0.374452005521614</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2980,7 +2980,7 @@
         <v>0.235262369481904</v>
       </c>
       <c r="B20" s="15" t="n">
-        <v>-0.501918248862394</v>
+        <v>-0.511327827898784</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>273</v>
@@ -2991,7 +2991,7 @@
         <v>0.215</v>
       </c>
       <c r="B21" s="15" t="n">
-        <v>-0.205037068416587</v>
+        <v>-0.295949617094494</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>274</v>
@@ -3002,7 +3002,7 @@
         <v>0.195</v>
       </c>
       <c r="B22" s="15" t="n">
-        <v>0.241357561487556</v>
+        <v>-0.0167794554956538</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>275</v>
@@ -3013,7 +3013,7 @@
         <v>0.175</v>
       </c>
       <c r="B23" s="15" t="n">
-        <v>0.993648164964695</v>
+        <v>0.361282974718848</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>276</v>
@@ -3021,7 +3021,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="16" t="n">
-        <v>0.160726656224811</v>
+        <v>0.1304559005772</v>
       </c>
       <c r="B24" s="15" t="n">
         <v>1.94</v>
@@ -3035,7 +3035,7 @@
         <v>0.15</v>
       </c>
       <c r="B25" s="15" t="n">
-        <v>3.16450389227658</v>
+        <v>1.06516066693947</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>278</v>
@@ -3096,7 +3096,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="15" t="n">
-        <v>0.32530642743704</v>
+        <v>0.0623803529555808</v>
       </c>
       <c r="E2" s="21" t="n">
         <f aca="false">Assumptions!$C$41</f>
@@ -3168,7 +3168,7 @@
       </c>
       <c r="D5" s="24" t="n">
         <f aca="false">SUMPRODUCT(D2:D4,$E$2:$E$4)</f>
-        <v>1.29023476484341</v>
+        <v>1.1982106387749</v>
       </c>
       <c r="E5" s="25" t="n">
         <f aca="false">SUM(E2:E4)</f>
@@ -5355,7 +5355,7 @@
         <v>16</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>0.115</v>
+        <v>0.05</v>
       </c>
       <c r="H35" s="2" t="s">
         <v>83</v>

</xml_diff>